<commit_message>
Regenerate demo packages in zh/en through the real packaging modules
</commit_message>
<xml_diff>
--- a/examples/demo_output/demo_sample/demo_sample.xlsx
+++ b/examples/demo_output/demo_sample/demo_sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表1_Sample_oxide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表1_Sample oxide composition" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -58,10 +58,10 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -425,16 +425,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="004472C4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>标题: Table 1 Sample oxide composition (synthetic)</t>
+          <t>标题: Sample oxide composition</t>
         </is>
       </c>
     </row>

</xml_diff>